<commit_message>
adding in online and hooking to the website
</commit_message>
<xml_diff>
--- a/ibokki_spell_cards.xlsx
+++ b/ibokki_spell_cards.xlsx
@@ -92,7 +92,7 @@
     <t xml:space="preserve">Ward Pulse</t>
   </si>
   <si>
-    <t xml:space="preserve">Each Ward you control gains 1 HP.</t>
+    <t xml:space="preserve">Each Ward you control gains 1 HP. If you control a Ward, deal 1 damage.</t>
   </si>
   <si>
     <t xml:space="preserve">Scales with Ward density. Weak early but synergizes with multi-Ward strategies at higher levels.</t>
@@ -665,7 +665,7 @@
     <t xml:space="preserve">Burning Hands</t>
   </si>
   <si>
-    <t xml:space="preserve">Deal 1 damage. Place 1 Burn marker on your opponent. (At the start of each of your opponent's turns, each Burn marker on them deals 1 damage. Burns expire at end of round.)</t>
+    <t xml:space="preserve">Deal 1 damage. Place 1 Burn marker on your opponent. (At the start of each of your opponent's turns, each Burn marker on them deals 1 damage; then one Burn marker is removed.)</t>
   </si>
   <si>
     <t xml:space="preserve">First Burn card establishes the keyword. DoT is Evocation's answer to Abjuration's slow defensive game — it ticks while the opponent is busy building Wards.</t>
@@ -695,7 +695,7 @@
     <t xml:space="preserve">Kindle</t>
   </si>
   <si>
-    <t xml:space="preserve">Place 2 Burn markers on your opponent.</t>
+    <t xml:space="preserve">Place 1 Burn marker on your opponent.</t>
   </si>
   <si>
     <t xml:space="preserve">EVO-007</t>
@@ -1319,7 +1319,7 @@
     <t xml:space="preserve">Foretell</t>
   </si>
   <si>
-    <t xml:space="preserve">Look at your opponent's hand.</t>
+    <t xml:space="preserve">Look at your opponent's hand. Deal 1 damage.</t>
   </si>
   <si>
     <t xml:space="preserve">Cheap information. Against a reactive Abjuration deck, knowing which counters they hold lets you sequence safely around them.</t>
@@ -1433,7 +1433,7 @@
     <t xml:space="preserve">Your opponent puts the top 2 cards of their Resource Deck into their discard pile.</t>
   </si>
   <si>
-    <t xml:space="preserve">Opens the alternate win condition — decking the opponent out. Slow but inevitable against a defensive deck that wants long rounds.</t>
+    <t xml:space="preserve">Accelerates the opponent’s exhaustion clock — every milled card brings their next reshuffle (and its escalating damage) closer.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-021</t>
@@ -1466,7 +1466,7 @@
     <t xml:space="preserve">Far Sight</t>
   </si>
   <si>
-    <t xml:space="preserve">Look at the top 3 cards of your opponent's Resource Deck. You may put one of them into their discard pile.</t>
+    <t xml:space="preserve">Look at the top 3 cards of your opponent's Resource Deck. You may put one of them into their discard pile. Deal 1 damage.</t>
   </si>
   <si>
     <t xml:space="preserve">Information and light mill in one. Strips an answer off the top before they ever see it.</t>
@@ -1538,7 +1538,7 @@
     <t xml:space="preserve">Shuffle your discard pile into your Resource Deck, then draw 2 cards.</t>
   </si>
   <si>
-    <t xml:space="preserve">Refills the whole deck mid-game — anti-deck-out insurance and a huge tempo reset. Against an Abjuration grind, you simply never run out.</t>
+    <t xml:space="preserve">A free reshuffle — resets your deck WITHOUT the exhaustion damage a forced recycle costs, then draws 2. Anti-mill and anti-exhaustion tech.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-029</t>
@@ -1727,7 +1727,7 @@
     <t xml:space="preserve">Your opponent shuffles their hand into their Resource Deck, then puts the top 8 cards of their Resource Deck into their discard pile.</t>
   </si>
   <si>
-    <t xml:space="preserve">The deck-out win condition made real. Against an Abjuration deck content to durdle behind Wards, this ends the game from the deck itself.</t>
+    <t xml:space="preserve">The mill haymaker — dumps 8 cards toward the opponent’s next exhaustion tick and scrambles their hand on the way.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-044</t>
@@ -2105,10 +2105,10 @@
     <t xml:space="preserve">Shuffle your discard pile into your Resource Deck.</t>
   </si>
   <si>
-    <t xml:space="preserve">Counter — Divination (mill / deck-out)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The anti-deck-out tech — refill so the mill plan can't close. Dead against a fast clock.</t>
+    <t xml:space="preserve">Counter — Divination (mill / exhaustion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anti-mill / anti-exhaustion tech — a free recycle that dodges the escalating reshuffle damage. Dead against a fast clock.</t>
   </si>
   <si>
     <t xml:space="preserve">GAM-017</t>
@@ -2150,7 +2150,7 @@
     <t xml:space="preserve">Counter / Complement — Mill</t>
   </si>
   <si>
-    <t xml:space="preserve">Free mill for any deck — supports a deck-out plan or pressures a fragile combo deck. Modest at 3 cards and one-per-turn.</t>
+    <t xml:space="preserve">Free mill for any deck — pushes the opponent toward their next exhaustion tick, or pressures a fragile combo deck. Modest at 3 cards and one-per-turn.</t>
   </si>
   <si>
     <t xml:space="preserve">GAM-020</t>
@@ -4163,7 +4163,7 @@
         <v>12</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>241</v>
@@ -4188,7 +4188,7 @@
         <v>12</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>241</v>
@@ -4294,7 +4294,7 @@
         <v>34</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>241</v>

</xml_diff>

<commit_message>
Div early-game buffs (Foretell, Anticipate) + tier-up bonus swap
Balance (user-approved; xlsx + cards.json + effects in sync):
- Foretell (DIV-011): deal 1 -> 2. Div's L1 damage axis - "Spark plus
  intel" for M. Eleven of Div's twelve L1 spells touch only your own
  deck; this gives the school early reach without out-racing Evo.
- Anticipate (DIV-014): draw 1 -> draw 1 and deal 1. Div's only L1
  reaction now actually threatens.

Rules: prepared-spell replacements are 2 (not 1) in rounds where the
level-up just raised your max castable spell level (L5 etc.) -
unlocking a new tier deserves more than one showcase slot.
replacementLimit() in levels.ts; Design_Doc ruling added.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ibokki_spell_cards.xlsx
+++ b/ibokki_spell_cards.xlsx
@@ -1319,7 +1319,7 @@
     <t xml:space="preserve">Foretell</t>
   </si>
   <si>
-    <t xml:space="preserve">Look at your opponent's hand. Deal 1 damage.</t>
+    <t xml:space="preserve">Look at your opponent's hand. Deal 2 damage.</t>
   </si>
   <si>
     <t xml:space="preserve">Cheap information. Against a reactive Abjuration deck, knowing which counters they hold lets you sequence safely around them.</t>
@@ -1355,7 +1355,7 @@
     <t xml:space="preserve">Anticipate</t>
   </si>
   <si>
-    <t xml:space="preserve">When your opponent casts a spell, draw 1 card.</t>
+    <t xml:space="preserve">When your opponent casts a spell, draw 1 card and deal 1 damage to them.</t>
   </si>
   <si>
     <t xml:space="preserve">You saw it coming. A Reaction that stops nothing — it simply converts the opponent's tempo into your card advantage.</t>

</xml_diff>

<commit_message>
changing the dynamic of the divination deck entirely to remove mill. I hate mill
</commit_message>
<xml_diff>
--- a/ibokki_spell_cards.xlsx
+++ b/ibokki_spell_cards.xlsx
@@ -1331,10 +1331,10 @@
     <t xml:space="preserve">Omen</t>
   </si>
   <si>
-    <t xml:space="preserve">Look at the top 4 cards of your Resource Deck. Put one Material (M) component from among them into your hand and the rest on the bottom in any order.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A focused dig that rewards a Material-dense deck. Finds the symbol you need while burying what you don't.</t>
+    <t xml:space="preserve">Prophecy - at the start of your opponent's second turn from now, deal 3 damage to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The L1 starter doom - gives the prophecy identity a presence in rounds 1-4 before the L2+ dooms unlock (m12 finding). One more than Foretell's sting because it arrives two turns late.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-013</t>
@@ -1430,10 +1430,10 @@
     <t xml:space="preserve">Foreclosure</t>
   </si>
   <si>
-    <t xml:space="preserve">Your opponent puts the top 2 cards of their Resource Deck into their discard pile.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accelerates the opponent’s exhaustion clock — every milled card brings their next reshuffle (and its escalating damage) closer.</t>
+    <t xml:space="preserve">Prophecy - at the start of your opponent's second turn from now, deal 4 damage to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The prophecy workhorse - a 4-damage doom on a 2-turn fuse. Announced pressure the opponent must plan around.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-021</t>
@@ -1466,10 +1466,10 @@
     <t xml:space="preserve">Far Sight</t>
   </si>
   <si>
-    <t xml:space="preserve">Look at the top 3 cards of your opponent's Resource Deck. You may put one of them into their discard pile. Deal 1 damage.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Information and light mill in one. Strips an answer off the top before they ever see it.</t>
+    <t xml:space="preserve">Look at the top 3 cards of your Resource Deck and put them back in any order. Prophecy - at the start of your opponent's next turn, deal 2 damage to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scry and doom in one - sculpts your next draws while a short-fuse prophecy lands next turn.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-024</t>
@@ -1538,7 +1538,7 @@
     <t xml:space="preserve">Shuffle your discard pile into your Resource Deck, then draw 2 cards.</t>
   </si>
   <si>
-    <t xml:space="preserve">A free reshuffle — resets your deck WITHOUT the exhaustion damage a forced recycle costs, then draws 2. Anti-mill and anti-exhaustion tech.</t>
+    <t xml:space="preserve">A free reshuffle - resets your deck WITHOUT the exhaustion damage a forced recycle costs, then draws 2. Anti-exhaustion tech.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-029</t>
@@ -1583,10 +1583,10 @@
     <t xml:space="preserve">Entropy</t>
   </si>
   <si>
-    <t xml:space="preserve">Your opponent puts the top 4 cards of their Resource Deck into their discard pile.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The mill plan's mid-game accelerant. Four cards a cast adds up fast against a slow deck that wants the game to go long.</t>
+    <t xml:space="preserve">Prophecy - at the start of your opponent's third turn from now, deal 7 damage to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The mid-game doom - 7 damage on a 3-turn fuse; cast early and every one of their turns becomes a countdown.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-033</t>
@@ -1724,10 +1724,10 @@
     <t xml:space="preserve">Oblivion</t>
   </si>
   <si>
-    <t xml:space="preserve">Your opponent shuffles their hand into their Resource Deck, then puts the top 8 cards of their Resource Deck into their discard pile.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The mill haymaker — dumps 8 cards toward the opponent’s next exhaustion tick and scrambles their hand on the way.</t>
+    <t xml:space="preserve">Prophecy - at the start of your opponent's third turn from now, deal 9 damage to them. This damage cannot be prevented or absorbed by Wards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The prophecy haymaker - 9 unwardable damage in 3 turns. Answer it at cast time or race it.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-044</t>
@@ -2105,10 +2105,10 @@
     <t xml:space="preserve">Shuffle your discard pile into your Resource Deck.</t>
   </si>
   <si>
-    <t xml:space="preserve">Counter — Divination (mill / exhaustion)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anti-mill / anti-exhaustion tech — a free recycle that dodges the escalating reshuffle damage. Dead against a fast clock.</t>
+    <t xml:space="preserve">Counter - Divination (prophecy / exhaustion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anti-exhaustion tech - a free recycle that dodges the escalating reshuffle damage. Dead against a fast clock.</t>
   </si>
   <si>
     <t xml:space="preserve">GAM-017</t>
@@ -2144,13 +2144,13 @@
     <t xml:space="preserve">Saboteur's Kit</t>
   </si>
   <si>
-    <t xml:space="preserve">Your opponent puts the top 3 cards of their Resource Deck into their discard pile.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Counter / Complement — Mill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Free mill for any deck — pushes the opponent toward their next exhaustion tick, or pressures a fragile combo deck. Modest at 3 cards and one-per-turn.</t>
+    <t xml:space="preserve">Prophecy - at the start of your opponent's second turn from now, deal 2 damage to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complement - Prophecy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A free time-bomb for any deck - 2 damage on a 2-turn fuse. Modest alone; stacked copies build a schedule of dooms.</t>
   </si>
   <si>
     <t xml:space="preserve">GAM-020</t>

</xml_diff>

<commit_message>
balancing changes and tests
</commit_message>
<xml_diff>
--- a/ibokki_spell_cards.xlsx
+++ b/ibokki_spell_cards.xlsx
@@ -68,7 +68,7 @@
     <t xml:space="preserve">S</t>
   </si>
   <si>
-    <t xml:space="preserve">Add 2 HP to a Ward you control. If you control no Ward, create one with 1 HP instead. Then remove 1 Burn marker from yourself.</t>
+    <t xml:space="preserve">Add 2 HP to a Ward you control. If you control no Ward, create one with 2 HP instead. Then remove 1 Burn marker from yourself.</t>
   </si>
   <si>
     <t xml:space="preserve">Good early-game Ward sustain. Rewards players who already established a Ward on a prior turn.</t>
@@ -116,10 +116,10 @@
     <t xml:space="preserve">Stone Stance</t>
   </si>
   <si>
-    <t xml:space="preserve">Until the end of the round, spell damage dealt to you is reduced by 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enables early Reaction spam by discounting the first one. Strong opener for a reactive game plan.</t>
+    <t xml:space="preserve">Until the end of the round, spell damage dealt to you is reduced by 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Round-long -2 to incoming spell damage - the anti-cantrip tax. Charges Reckoning while it blunts aggro; near-irrelevant against big single hits.</t>
   </si>
   <si>
     <t xml:space="preserve">ABJ-006</t>
@@ -461,7 +461,7 @@
     <t xml:space="preserve">Reckoning</t>
   </si>
   <si>
-    <t xml:space="preserve">Deal damage to your opponent equal to the total amount of damage you have prevented this round.</t>
+    <t xml:space="preserve">Deal damage to your opponent equal to half the total damage you have prevented this match, rounded up. Damage your Wards absorb counts as prevented.</t>
   </si>
   <si>
     <t xml:space="preserve">Rewards a patient defensive game — the more attacks you've weathered and mitigated, the harder this hits. Pairs naturally with Absorb and other prevention effects to set up a large burst in the same round.</t>
@@ -1211,10 +1211,10 @@
     <t xml:space="preserve">Foresight</t>
   </si>
   <si>
-    <t xml:space="preserve">Look at the top 3 cards of your Resource Deck. Put one into your hand and the rest back on top in any order.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Selection over raw draw. Smooths your next two turns and stacks the top of your deck for Premonition or Calculated Draw.</t>
+    <t xml:space="preserve">Look at the top 3 cards of your Resource Deck. Put one into your hand and the rest back on top in any order. Until the end of the round, spell damage dealt to you is reduced by 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selection plus the foreseen-blow flinch - a round-long -1 against chip damage. The seer's early answer to cantrip aggro.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-003</t>
@@ -1223,10 +1223,10 @@
     <t xml:space="preserve">Divine</t>
   </si>
   <si>
-    <t xml:space="preserve">Look at the top 2 cards of your Resource Deck. Put one into your hand and the other on the bottom.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cheap filtering. Trades a little card economy for the guarantee that you keep the piece you actually need.</t>
+    <t xml:space="preserve">Look at the top 2 cards of your Resource Deck. Put one into your hand and the other on the bottom. Then remove 1 Burn marker from yourself.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheap filtering that also shrugs off a Burn you saw coming. The rider is a pure Evocation tax - dead by design against burn-less schools.</t>
   </si>
   <si>
     <t xml:space="preserve">DIV-004</t>
@@ -3469,7 +3469,7 @@
         <v>3</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>145</v>
@@ -5507,7 +5507,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>390</v>
+        <v>447</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>435</v>

</xml_diff>

<commit_message>
cards + engine + sim: the ledger family — ABJ-046/047/048 spend the Reckoning bank
Warding Tithe (S L1: spend <=4 -> that big a Ward), Sealed Verdict (S L2
Reaction: spend 6 -> cancel target spell), Restoring Rune (S L2: spend <=6
-> heal half). New spendPrevented context op is the first and only
decrementer of damagePreventedTotal — Reckoning's text untouched, its
payload now competes with tempo. Sub-minimum casts whiff-guarded
(LEDGER_MIN, both legality paths); bots price the spenders via
stored-value payload terms + Verdict rides the doom-aware armed-cancel
valuation. Authored in the xlsx as inlineStr rows; 6 new engine tests.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ibokki_spell_cards.xlsx
+++ b/ibokki_spell_cards.xlsx
@@ -2572,7 +2572,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -3828,6 +3828,129 @@
       <c r="H46" s="6"/>
       <c r="I46" s="5" t="s">
         <v>200</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>ABJ-046</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Warding Tithe</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Abjuration</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Spell</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Spend up to 4 of the damage you have prevented this match. Create a Ward with HP equal to the amount spent.</t>
+        </is>
+      </c>
+      <c r="H47" s="6"/>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Ledger family (2026-08-13). Spends the Reckoning bank for tempo - every point spent is a point the late nuke loses. Gives prevention a use against doom decks that never touch wards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>ABJ-047</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Sealed Verdict</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Abjuration</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Spend 6 of the damage you have prevented this match: cancel target spell. Castable only while you have at least 6 prevented.</t>
+        </is>
+      </c>
+      <c r="H48" s="6"/>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Ledger family. A cancel funded by the bank instead of scarce attached fuel - the extra answer per round Abjuration lacked against multi-doom turns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>ABJ-048</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Restoring Rune</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Abjuration</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Spell</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Spend up to 6 of the damage you have prevented this match. Heal half the amount spent, rounded down.</t>
+        </is>
+      </c>
+      <c r="H49" s="6"/>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Ledger family. Sustain option - trades future Reckoning payload for present HP.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cards + client: exp-9 Evo tune + prevention-ledger HUD
- EVO-006 Kindle -> Stoke: burn marker replaced by V-component recursion
  (return up to 2 Verbal-providing cards from discard)
- EVO-011 damage 4 -> 5; L2 anchor damage 5 -> 6
- Evo M-cancel now also hits Reactions (parity with Counterbind's scope)
- client HUD: surface damagePreventedTotal as a public seal segment on the
  player plate — m55's invisible 35-damage Reckoning felt like a cheat;
  the ledger funds Reckoning/Tithe/Verdict/Rune and is already public data

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ibokki_spell_cards.xlsx
+++ b/ibokki_spell_cards.xlsx
@@ -692,10 +692,10 @@
     <t xml:space="preserve">EVO-006</t>
   </si>
   <si>
-    <t xml:space="preserve">Kindle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Place 1 Burn marker on your opponent.</t>
+    <t xml:space="preserve">Stoke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Return up to two Verbal-providing component cards from your discard pile to your hand.</t>
   </si>
   <si>
     <t xml:space="preserve">EVO-007</t>
@@ -752,7 +752,7 @@
     <t xml:space="preserve">VV</t>
   </si>
   <si>
-    <t xml:space="preserve">Deal 4 damage to your opponent.</t>
+    <t xml:space="preserve">Deal 5 damage to your opponent.</t>
   </si>
   <si>
     <t xml:space="preserve">EVO-012</t>
@@ -815,7 +815,7 @@
     <t xml:space="preserve">Fireball</t>
   </si>
   <si>
-    <t xml:space="preserve">Deal 5 damage to your opponent.</t>
+    <t xml:space="preserve">Deal 6 damage to your opponent.</t>
   </si>
   <si>
     <t xml:space="preserve">Iconic spell at iconic cost. Anchors the L2 power curve.</t>
@@ -956,7 +956,7 @@
     <t xml:space="preserve">Mana Burn</t>
   </si>
   <si>
-    <t xml:space="preserve">Cancel target spell that requires a Material (M) component. Deal 2 damage to your opponent.</t>
+    <t xml:space="preserve">Cancel target spell or Reaction that requires a Material (M) component. Deal 2 damage to your opponent.</t>
   </si>
   <si>
     <t xml:space="preserve">The Evocation parallel to Counterbind — same anti-school role but with damage tacked on rather than pure denial.</t>

</xml_diff>